<commit_message>
feat: alinhar simulador barter com planilha Simulador_CashBack_Barter_2026
- Atualizar nomenclatura para Preco Pedido PRAZO, Preco Pedido BARTER Cash Back equivalente e Total Retorno
- Calcular Incentivo Barter % e $, Cash Back e Volume TROCA equivalencia
- Refatorar tabela do Racional com todas as etapas da planilha de 2026
- Remover termo Seguro Agricola mantendo garantia exclusivamente como CPR Fisica
- Tratar despesa de deslocamento de frete de forma unitaria sobre o Preco Livre
</commit_message>
<xml_diff>
--- a/Simulador_CashBack_Barter_2026.xlsx
+++ b/Simulador_CashBack_Barter_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e0e760a1110f3163/Projetos/Barter Simulator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{4471872B-2932-4B94-9F5A-F15A4FAF387F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFECC2ED-E5F5-42E4-8D98-4CFF7DB18D9C}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{4471872B-2932-4B94-9F5A-F15A4FAF387F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D64259F7-1C74-43DB-98BB-10B401364033}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{507E8C52-4AC5-4303-BA21-5B7B491348B3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{507E8C52-4AC5-4303-BA21-5B7B491348B3}"/>
   </bookViews>
   <sheets>
     <sheet name="R.T._usd" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="60">
   <si>
     <t>NUTRADE</t>
   </si>
@@ -379,6 +379,32 @@
   </si>
   <si>
     <t>SIM</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Preço </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Commodity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Livre (adicionar KM chão e terra)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -444,7 +470,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -484,6 +510,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -582,7 +614,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -698,6 +730,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1182,7 +1217,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="62" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="5">
@@ -1220,7 +1255,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="61" t="s">
         <v>47</v>
       </c>
       <c r="B3" s="32">
@@ -1284,7 +1319,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="16.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="61" t="s">
         <v>50</v>
       </c>
       <c r="B5" s="5">
@@ -1451,7 +1486,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="B12" s="13">
         <f>B11-IF(B9="SIM",(B11*0.2%+0.6),0)</f>
@@ -1475,7 +1510,7 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="61" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="14">
@@ -1543,7 +1578,7 @@
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="61" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="38">
@@ -1567,7 +1602,7 @@
       <c r="K16" s="28"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="61" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="16">
@@ -1754,7 +1789,7 @@
       <c r="K24" s="28"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="61" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="22">
@@ -1774,7 +1809,7 @@
       <c r="K25" s="28"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="61" t="s">
         <v>26</v>
       </c>
       <c r="B26" s="5">
@@ -1871,7 +1906,7 @@
       <c r="K29" s="27"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="61" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="19">
@@ -1923,7 +1958,7 @@
       <c r="K31" s="27"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="61" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="20">
@@ -1956,7 +1991,7 @@
       <c r="K32" s="27"/>
     </row>
     <row r="33" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="63" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="23">
@@ -2037,7 +2072,7 @@
       <formula>$C$32</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9 E9" xr:uid="{535578D5-9BE4-4936-9ABF-3856D88A47DD}">
       <formula1>"SIM,NÃO"</formula1>
     </dataValidation>

</xml_diff>